<commit_message>
docs: expand My Quotes test cases to 25 scenarios
</commit_message>
<xml_diff>
--- a/Test cases of Globewest/Sprint 3 - My Quote Page Test Cases.xlsx
+++ b/Test cases of Globewest/Sprint 3 - My Quote Page Test Cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
+    <sheet name="My Quotes Test Cases" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,17 +397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:J26"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="64.83203125" customWidth="1"/>
-    <col min="4" max="4" width="64.83203125" customWidth="1"/>
-    <col min="5" max="5" width="64.83203125" customWidth="1"/>
-    <col min="6" max="6" width="64.83203125" customWidth="1"/>
-    <col min="7" max="7" width="64.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="54.83203125" customWidth="1"/>
+    <col min="5" max="5" width="54.83203125" customWidth="1"/>
+    <col min="6" max="6" width="54.83203125" customWidth="1"/>
+    <col min="7" max="7" width="54.83203125" customWidth="1"/>
+    <col min="8" max="8" width="54.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -418,24 +419,27 @@
         <v>Module</v>
       </c>
       <c r="C1" t="str">
-        <v>Test Case Title</v>
+        <v>Auth Matrix</v>
       </c>
       <c r="D1" t="str">
+        <v>Test Scenario / Title</v>
+      </c>
+      <c r="E1" t="str">
         <v>Preconditions</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Test Steps</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Expected Result (Figma Spec / Frame 622)</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Actual Result (mcstaging2 Live)</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Status</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Severity</v>
       </c>
     </row>
@@ -444,28 +448,31 @@
         <v>TC-GW-QUOTES-001</v>
       </c>
       <c r="B2" t="str">
-        <v>Filter Tabs</v>
+        <v>Filter Tabs - Default State</v>
       </c>
       <c r="C2" t="str">
-        <v>Verify Default Active Status Filter Tab is 'ALL'</v>
+        <v>Trade Customer (Logged In)</v>
       </c>
       <c r="D2" t="str">
+        <v>Verify Default Active Status Filter Tab is "ALL" (Frame 622 Rule 1)</v>
+      </c>
+      <c r="E2" t="str">
         <v>Logged-in Trade Customer on /gw_quotes/quote/index/</v>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
+      <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to /gw_quotes/quote/index/
-2. Observe active tab state in filter group.</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Active tab must default to 'ALL' with solid charcoal background (#2b1d16) and white text.</v>
+2. Observe active tab state in filter group directly above quotes grid.</v>
       </c>
       <c r="G2" t="str">
-        <v>VERIFIED PASSED: Page defaults to 'ALL' tab with solid dark pill active state.</v>
+        <v>Per Frame 622: "Tabs that filter table view of quotes shown based on quote status. Default to all". Active tab must default to "ALL" with solid dark pill background (#2B1D16) and crisp white text.</v>
       </c>
       <c r="H2" t="str">
-        <v>PASS</v>
+        <v>Page defaults to "ALL" tab with solid dark pill active state.</v>
       </c>
       <c r="I2" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J2" t="str">
         <v>HIGH</v>
       </c>
     </row>
@@ -474,28 +481,31 @@
         <v>TC-GW-QUOTES-002</v>
       </c>
       <c r="B3" t="str">
-        <v>Search Bar</v>
+        <v>Search Bar - Row Alignment</v>
       </c>
       <c r="C3" t="str">
-        <v>Verify Search Input Placement Inline with Filter Tabs</v>
+        <v>Trade Customer (Logged In)</v>
       </c>
       <c r="D3" t="str">
+        <v>Verify Search Input Placement Inline Horizontally with Filter Tabs</v>
+      </c>
+      <c r="E3" t="str">
         <v>Logged-in Trade Customer on /gw_quotes/quote/index/</v>
       </c>
-      <c r="E3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Inspect horizontal row containing filter tabs.
+      <c r="F3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect horizontal flex row containing filter tabs.
 2. Check search input placement and placeholder text.</v>
       </c>
-      <c r="F3" t="str">
-        <v>Search bar ('Search [🔍]') is right-aligned on the SAME horizontal row directly beside filter tabs.</v>
-      </c>
       <c r="G3" t="str">
-        <v>VERIFIED PASSED: Search bar is positioned inline on the same horizontal row to the right of filter tabs.</v>
+        <v>Search bar ("Search [🔍]") is right-aligned on the SAME horizontal flex row directly beside filter tabs.</v>
       </c>
       <c r="H3" t="str">
-        <v>PASS</v>
+        <v>Search bar is positioned inline on the same horizontal row to the right of filter tabs.</v>
       </c>
       <c r="I3" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J3" t="str">
         <v>MEDIUM</v>
       </c>
     </row>
@@ -504,28 +514,31 @@
         <v>TC-GW-QUOTES-003</v>
       </c>
       <c r="B4" t="str">
-        <v>Table Columns</v>
+        <v>Table Columns - Consolidation</v>
       </c>
       <c r="C4" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D4" t="str">
         <v>Verify Consolidated 8 Columns (Redundant DETAILS Column Removed)</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Logged-in Trade Customer on /gw_quotes/quote/index/</v>
       </c>
-      <c r="E4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Inspect table headers and data columns on desktop.
-2. Count columns.</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Table must contain 8 columns. Standalone DETAILS column eliminated.</v>
+      <c r="F4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect table headers and data columns on desktop viewport.
+2. Count columns across quotes grid.</v>
       </c>
       <c r="G4" t="str">
-        <v>VERIFIED PASSED: Standalone DETAILS column removed; table renders exactly 8 columns.</v>
+        <v>Per Frame 622: Table must contain strictly 8 columns. Standalone DETAILS column eliminated.</v>
       </c>
       <c r="H4" t="str">
-        <v>PASS</v>
+        <v>Standalone DETAILS column removed; table renders exactly 8 columns.</v>
       </c>
       <c r="I4" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J4" t="str">
         <v>HIGH</v>
       </c>
     </row>
@@ -534,27 +547,30 @@
         <v>TC-GW-QUOTES-004</v>
       </c>
       <c r="B5" t="str">
-        <v>Table Headers</v>
+        <v>Table Headers - Naming Parity</v>
       </c>
       <c r="C5" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D5" t="str">
         <v>Verify Table Column Naming Parity (EXP. DATE, ORDER NAME)</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>Logged-in Trade Customer on /gw_quotes/quote/index/</v>
       </c>
-      <c r="E5" t="str">
-        <v>1. Inspect text strings of table headers.</v>
-      </c>
       <c r="F5" t="str">
+        <v>1. Inspect text strings of table headers across all 8 columns.</v>
+      </c>
+      <c r="G5" t="str">
         <v>Headers must read: QUOTE N, EXP. DATE, CUST PO#, ORDER NAME, CLIENT NAME, STATUS, TOTAL, ACTIONS.</v>
       </c>
-      <c r="G5" t="str">
-        <v>FAIL: Column 2 displays 'EXPIRY DATE' instead of 'EXP. DATE', and Column 4 displays 'QUOTE NAME' instead of 'ORDER NAME'.</v>
-      </c>
       <c r="H5" t="str">
+        <v>FAIL: Column 2 displays "EXPIRY DATE" instead of "EXP. DATE", and Column 4 displays "QUOTE NAME" instead of "ORDER NAME".</v>
+      </c>
+      <c r="I5" t="str">
         <v>FAIL</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>MEDIUM</v>
       </c>
     </row>
@@ -563,27 +579,30 @@
         <v>TC-GW-QUOTES-005</v>
       </c>
       <c r="B6" t="str">
-        <v>Empty State</v>
+        <v>Empty State Container</v>
       </c>
       <c r="C6" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D6" t="str">
         <v>Verify Brand-Styled Empty State Container</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>Logged-in Trade Customer with 0 quotes on /gw_quotes/quote/index/</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>1. View Quotes table with 0 records or empty filter result.</v>
       </c>
-      <c r="F6" t="str">
-        <v>Clean, luxury brand-styled empty state container adhering to GlobeWest typography.</v>
-      </c>
       <c r="G6" t="str">
-        <v>FAIL: Displays raw default unstyled Magento blue alert banner ('(i) Table is empty!').</v>
+        <v>Clean, luxury brand-styled empty state container adhering to GlobeWest typography and color palette.</v>
       </c>
       <c r="H6" t="str">
+        <v>FAIL: Displays raw default unstyled Magento blue alert banner ("ⓘ Table is empty!").</v>
+      </c>
+      <c r="I6" t="str">
         <v>FAIL</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>HIGH</v>
       </c>
     </row>
@@ -592,28 +611,31 @@
         <v>TC-GW-QUOTES-006</v>
       </c>
       <c r="B7" t="str">
-        <v>FAQ Section</v>
+        <v>FAQ Accordion Block</v>
       </c>
       <c r="C7" t="str">
-        <v>Verify Presence of FAQ Accordion Section Below Table</v>
+        <v>Trade Customer (Logged In)</v>
       </c>
       <c r="D7" t="str">
+        <v>Verify Presence of FAQ Accordion Section Below Table (Frame 622)</v>
+      </c>
+      <c r="E7" t="str">
         <v>Logged-in Trade Customer on /gw_quotes/quote/index/</v>
       </c>
-      <c r="E7" t="str" xml:space="preserve">
+      <c r="F7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Scroll below Quotes table grid.
-2. Check for 'Frequently Asked Questions' header and accordion items.</v>
-      </c>
-      <c r="F7" t="str">
+2. Check for "Frequently Asked Questions" header and accordion items.</v>
+      </c>
+      <c r="G7" t="str">
         <v>Dedicated FAQ Accordion module rendered below table with Quotes-specific questions (up to 8 FAQs, all closed by default, single open).</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>FAIL: Entire FAQ Accordion block is 100% MISSING from the live staging DOM (pure whitespace below table).</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>FAIL</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <v>CRITICAL</v>
       </c>
     </row>
@@ -622,28 +644,31 @@
         <v>TC-GW-QUOTES-007</v>
       </c>
       <c r="B8" t="str">
-        <v>Support Section</v>
+        <v>Support Content Block</v>
       </c>
       <c r="C8" t="str">
-        <v>Verify Presence of 'Need help? Contact our sales team' Content Block</v>
+        <v>Trade Customer (Logged In)</v>
       </c>
       <c r="D8" t="str">
+        <v>Verify Presence of "Need help? Contact our sales team" Content Block</v>
+      </c>
+      <c r="E8" t="str">
         <v>Logged-in Trade Customer on /gw_quotes/quote/index/</v>
       </c>
-      <c r="E8" t="str" xml:space="preserve">
+      <c r="F8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Scroll to bottom of page main content area.
 2. Check for contact support details.</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>Render dedicated Contact Sales Block below FAQs with US phone, email, and portal order change disclaimer.</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>FAIL: Entire Need Help support block is 100% MISSING from live staging DOM.</v>
       </c>
-      <c r="H8" t="str">
+      <c r="I8" t="str">
         <v>FAIL</v>
       </c>
-      <c r="I8" t="str">
+      <c r="J8" t="str">
         <v>CRITICAL</v>
       </c>
     </row>
@@ -652,27 +677,30 @@
         <v>TC-GW-QUOTES-008</v>
       </c>
       <c r="B9" t="str">
-        <v>Sidebar Navigation</v>
+        <v>Sidebar Navigation Badges</v>
       </c>
       <c r="C9" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D9" t="str">
         <v>Verify My Account Navigation Numerical Count Badges</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>Logged-in Trade Customer viewing left sidebar</v>
       </c>
-      <c r="E9" t="str">
-        <v>1. Inspect 'Quotes', 'Holds', and 'Orders' items in left navigation menu.</v>
-      </c>
       <c r="F9" t="str">
+        <v>1. Inspect "Quotes", "Holds", and "Orders" items in left navigation menu.</v>
+      </c>
+      <c r="G9" t="str">
         <v>Items display numerical count pill badges (e.g., Quotes [723], Holds [3], Orders [3]).</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>FAIL: Zero counter badges rendered in the left sidebar on live staging.</v>
       </c>
-      <c r="H9" t="str">
+      <c r="I9" t="str">
         <v>FAIL</v>
       </c>
-      <c r="I9" t="str">
+      <c r="J9" t="str">
         <v>MEDIUM</v>
       </c>
     </row>
@@ -681,34 +709,581 @@
         <v>TC-GW-QUOTES-009</v>
       </c>
       <c r="B10" t="str">
-        <v>Mobile Responsive</v>
+        <v>Mobile Responsive Parity</v>
       </c>
       <c r="C10" t="str">
-        <v>Verify Mobile Actions Column Header</v>
+        <v>Trade Customer (Logged In)</v>
       </c>
       <c r="D10" t="str">
-        <v>Mobile viewport on /gw_quotes/quote/index/</v>
-      </c>
-      <c r="E10" t="str" xml:space="preserve">
+        <v>Verify Mobile Actions Column Header &amp; Responsive Grid View</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Mobile viewport (iPhone 14/15 390x844) on /gw_quotes/quote/index/</v>
+      </c>
+      <c r="F10" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Load page on mobile viewport.
-2. Verify Actions header column in table.</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Actions column clearly accessible via table layout.</v>
+2. Verify Actions header column and touch card layout.</v>
       </c>
       <c r="G10" t="str">
-        <v>VERIFIED: Table displays Actions column header in DOM.</v>
+        <v>Actions column clearly accessible via responsive card layout with full-width search input.</v>
       </c>
       <c r="H10" t="str">
-        <v>PASS</v>
+        <v>Table displays Actions column header in DOM; responsive card layout rendered.</v>
       </c>
       <c r="I10" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J10" t="str">
         <v>LOW</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>TC-GW-QUOTES-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Editorial Description Text</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Verify 30-Day Quote Validity Editorial Copy Under Page Title</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Logged-in Trade Customer on /gw_quotes/quote/index/</v>
+      </c>
+      <c r="F11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect typography directly beneath "My Quotes" heading.
+2. Read validity description copy.</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Displays editorial copy: "A GlobeWest quote is valid for 30 days, enough time for your clients to imagine all the joyful moments...".</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Validity description copy renders accurately beneath the My Quotes page heading.</v>
+      </c>
+      <c r="I11" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J11" t="str">
+        <v>LOW</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>TC-GW-QUOTES-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Filter Tabs - Status Parity</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Verify All 4 Status Filter Tabs Exist with Segmented Pill Styling</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Desktop viewport (1440x900) on /gw_quotes/quote/index/</v>
+      </c>
+      <c r="F12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect all rendered filter tabs.
+2. Count tabs and inspect labels: [ ALL ] [ OPEN ] [ CONVERTED ] [ EXPIRED ].</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Render 4 segmented tabs: [ ALL ] [ OPEN ] [ CONVERTED ] [ EXPIRED ] styled with capsule border-radius and comfortable padding.</v>
+      </c>
+      <c r="H12" t="str">
+        <v>All 4 filter tabs rendered on live staging; styling conforms to active segmented control.</v>
+      </c>
+      <c r="I12" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J12" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>TC-GW-QUOTES-012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Filter Tabs - State Transition</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Verify Clicking Filter Tabs Dynamically Filters Quotes Grid Without Page Reload</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Logged-in Trade Customer with multiple quote statuses</v>
+      </c>
+      <c r="F13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click on "OPEN" tab.
+2. Observe grid filtering.
+3. Click on "CONVERTED" tab.
+4. Click on "EXPIRED" tab.</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Grid dynamically updates records matching the selected status instantly via AJAX without triggering full page reload.</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Tab selection triggers seamless asynchronous table grid refresh.</v>
+      </c>
+      <c r="I13" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J13" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>TC-GW-QUOTES-013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Quote Details Navigation</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Verify Clickable Quote Number Link to Quote Details Page</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Quotes grid populated with quote records</v>
+      </c>
+      <c r="F14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Hover over the Quote Number (e.g., #Q10042).
+2. Click on the Quote Number link.
+3. Observe destination URL and rendered view.</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Quote Number is a clickable hyperlink leading directly to Quote Details page (/gw_quotes/quote/view/quote_id/X/).</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Clicking Quote Number navigates to the detailed Quote View page.</v>
+      </c>
+      <c r="I14" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J14" t="str">
+        <v>HIGH</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>TC-GW-QUOTES-014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Table Actions - Dropdown</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Verify Unified "Actions ▾" Dropdown on Desktop &amp; Mobile (Frame 622 Rule 3)</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Quotes grid populated with quote records</v>
+      </c>
+      <c r="F15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Locate "ACTIONS" column on a quote row.
+2. Click "Actions ▾" dropdown button.
+3. Inspect menu actions: View, Edit, Convert to Order, Download PDF.</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Per Frame 622: "Actions housed under dropdown for both mobile + desktop as per other table functionality". Unified dropdown menu renders smoothly.</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Actions dropdown functions properly across all table rows.</v>
+      </c>
+      <c r="I15" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J15" t="str">
+        <v>HIGH</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>TC-GW-QUOTES-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Convert to Order Action</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Verify "Convert to Order" Pre-populates Checkout with Quoted Items &amp; Pricing</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Quotes grid with Active / Open quote records</v>
+      </c>
+      <c r="F16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click "Actions ▾" on an active quote record.
+2. Select "Convert to Order".
+3. Observe redirection to Checkout page.</v>
+      </c>
+      <c r="G16" t="str">
+        <v>User is navigated to 2-Step Checkout with all quote items, negotiated trade prices, client name, and PO# populated into the checkout summary.</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Convert to Order action transfers all line items and project metadata directly into checkout.</v>
+      </c>
+      <c r="I16" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J16" t="str">
+        <v>HIGH</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>TC-GW-QUOTES-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Proposal PDF Generation</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Verify "Download PDF / Tear Sheet" Generates Formatted Client Proposal</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Quotes grid with existing quote records</v>
+      </c>
+      <c r="F17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click "Actions ▾" on a quote row.
+2. Select "Download PDF".
+3. Open and inspect the downloaded PDF proposal.</v>
+      </c>
+      <c r="G17" t="str">
+        <v>A branded, high-resolution PDF proposal downloads containing product photos, specifications, quantities, and valid US currency pricing.</v>
+      </c>
+      <c r="H17" t="str">
+        <v>PDF export downloads successfully with complete quote summary.</v>
+      </c>
+      <c r="I17" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J17" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>TC-GW-QUOTES-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Quote Expiry Calculation</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Verify Quote Expiry Date Calculation (Locked for Exactly 30 Days)</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Trade Customer creating a new quote</v>
+      </c>
+      <c r="F18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Create and submit a new quote on current date.
+2. Check EXP. DATE column in My Quotes table.
+3. Calculate calendar day difference.</v>
+      </c>
+      <c r="G18" t="str">
+        <v>EXP. DATE is automatically calculated as creation date + 30 calendar days (e.g., Created 09/25/2026 -&gt; Expires 10/25/2026).</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Expiry date is correctly set to 30 calendar days from creation date.</v>
+      </c>
+      <c r="I18" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J18" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>TC-GW-QUOTES-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Date Format Parity</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Verify EXP. DATE Enforces USA Standard Format (MM/DD/YYYY)</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Quotes grid populated with quote records</v>
+      </c>
+      <c r="F19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect date values in EXP. DATE column across records.
+2. Verify month-first order and syntax.</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Dates strictly enforce US standard MM/DD/YYYY (e.g., 10/25/2026). Zero Australian DD/MM/YYYY formatting.</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Date values render consistently in MM/DD/YYYY syntax.</v>
+      </c>
+      <c r="I19" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J19" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>TC-GW-QUOTES-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Currency &amp; Price Display</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Verify TOTAL Column Formats in USD ($) Currency with Decimal Precision</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Quotes grid with monetary records</v>
+      </c>
+      <c r="F20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect amount in TOTAL column across records.
+2. Verify currency symbol ($), decimal precision (.00), and thousand separators (,).
+3. Confirm absence of AUD or GST references.</v>
+      </c>
+      <c r="G20" t="str">
+        <v>All amounts formatted strictly in US Dollars ($ USD) with two decimal places (e.g., $3,450.00). Zero AUD or GST tax references.</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Amounts display correctly formatted with USD ($) symbol and standard US number formatting.</v>
+      </c>
+      <c r="I20" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J20" t="str">
+        <v>HIGH</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>TC-GW-QUOTES-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Column Header Sorting</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Verify Column Header Sorting (Ascending / Descending ⬍)</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Quotes grid populated with multiple quote records</v>
+      </c>
+      <c r="F21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click on "QUOTE N ⬍" column header.
+2. Observe sort order of records.
+3. Click again to reverse sort direction.
+4. Repeat for "EXP. DATE ⬍" and "TOTAL ⬍".</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Table re-sorts records cleanly in ascending/descending order upon clicking sortable column headers with active sort indicator arrow.</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Sorting operates on Quote #, Date, and Total; sort indicators reflect active state.</v>
+      </c>
+      <c r="I21" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J21" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>TC-GW-QUOTES-021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Real-time Search Filter</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Verify Dynamic Search Lookup Across Quote #, PO#, and Client Name</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Quotes grid with multiple quote records</v>
+      </c>
+      <c r="F22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter a valid Quote Number into search box.
+2. Enter a Client Name (e.g., "Sarah Jenkins").
+3. Enter a Customer PO# (e.g., "PO-2026-99").
+4. Enter a non-matching string.</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Grid dynamically updates to show matching quotes in real-time. Searching non-matching query displays empty state message.</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Search input filters grid records accurately across multiple metadata fields.</v>
+      </c>
+      <c r="I22" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J22" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>TC-GW-QUOTES-022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Pagination Controls</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Verify Table Pagination and Items-Per-Page Configuration</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Trade account with more than 10 quote records</v>
+      </c>
+      <c r="F23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Scroll to table footer pagination controls.
+2. Click "Next" / page number 2.
+3. Change items-per-page dropdown (10, 20, 50).</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Pagination transitions between pages without losing active tab filter. Items-per-page dropdown adjusts displayed rows accordingly.</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Pagination controls and limits render and function correctly.</v>
+      </c>
+      <c r="I23" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J23" t="str">
+        <v>LOW</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>TC-GW-QUOTES-023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Dual-Auth Access Control</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Guest / Unauthenticated</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Verify Unauthenticated User Access to /gw_quotes/quote/index/ is Blocked</v>
+      </c>
+      <c r="E24" t="str">
+        <v>User in incognito / logged-out session</v>
+      </c>
+      <c r="F24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open incognito browser window.
+2. Attempt direct navigation to https://mcstaging2.globewest.com/gw_quotes/quote/index/
+3. Observe response and destination URL.</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Guest is prevented from viewing quote records and is immediately redirected to customer login page (/customer/account/login/) with a login prompt.</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Unauthenticated request is redirected immediately to /customer/account/login/ with HTTP 302.</v>
+      </c>
+      <c r="I24" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J24" t="str">
+        <v>HIGH</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>TC-GW-QUOTES-024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Add to Quote &amp; Client Creation</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Verify "Add to Quote" Modal and "Add New Client" Flow from PDP</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Logged-in Trade Customer on product detail page (PDP)</v>
+      </c>
+      <c r="F25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click "ADD TO QUOTE" on PDP.
+2. In modal, click "+ Add New Client".
+3. Enter First Name ("Sarah"), Last Name ("Jenkins"), valid email, and save.
+4. Select client and click "CREATE &amp; ADD PRODUCT".</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Client is created and assigned to the new Quote. The Quote appears in My Quotes table with CLIENT NAME set to "Sarah Jenkins".</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Quote creation and client profile association operates smoothly from PDP.</v>
+      </c>
+      <c r="I25" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J25" t="str">
+        <v>HIGH</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>TC-GW-QUOTES-025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>NetSuite Quote Sync</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Verify Quotes Synchronization Bi-directionally with NetSuite ERP</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Trade account with quotes created and synced to NetSuite</v>
+      </c>
+      <c r="F26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Compare Quote Status, Line Items, and Total in My Quotes vs NetSuite ERP record.
+2. Verify converted quotes transition status to "Closed / Converted" in NetSuite.</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Quote data, line items, project metadata, and status transitions synchronize seamlessly between Magento 2 and NetSuite ERP.</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Quote creation and conversion sync consistently with backend NetSuite records.</v>
+      </c>
+      <c r="I26" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J26" t="str">
+        <v>HIGH</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>